<commit_message>
Refactor bullet scanning logic and update various Excel files
- Improved the bullet filtering logic in `checks_nedlagda.py` to better handle edge cases related to course names.
- Updated multiple Excel files across different directories, including:
  - Betygsrapportering.xlsx
  - Betygsskalor.xlsx
  - Bloom-taxonomi.xlsx
  - Examinationsformer.xlsx
  - Frasningskonsistens.xlsx
  - Färkunskapskrav.xlsx
  - Introfras.xlsx
  - Nedlagda kursreferenser.xlsx
  - Omfång på lärandemål.xlsx
  - Programkurser olänkade.xlsx
  - Samstämmighet svenska och engelska.xlsx
  - Stavfel och språkbruk.xlsx
  - Övrigt.xlsx
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/02 IHV/Analys/Programkurser olänkade.xlsx
+++ b/vault-dalarna-university/02 IHV/Analys/Programkurser olänkade.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Programkurser olänkade" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Programkurser olänkade'!$A$1:$E$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Programkurser olänkade'!$A$1:$E$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -526,7 +526,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>VBSKA</t>
+          <t>VGSEA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -536,24 +536,24 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Kursraden ser avbruten/feltrycklig ut</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>`) kurser som krävs för magisterexamen` (60 hp); rad: - ) kurser som krävs för magisterexamen, 60 hp</t>
+          <t>`Strategier för implementering av förbättringsarbete i hälso-sjukvård` (7,5 hp); rad: - Strategier för implementering av förbättringsarbete i hälso-sjukvård, 7,5 hp</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VBSKA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VGSEA</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>VGSEA</t>
+          <t>VIDRG</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -568,19 +568,19 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>`Strategier för implementering av förbättringsarbete i hälso-sjukvård` (7,5 hp); rad: - Strategier för implementering av förbättringsarbete i hälso-sjukvård, 7,5 hp</t>
+          <t>`Media och kommunikation inom idrott` (7,5hp); rad: - Media och kommunikation inom idrott, 7,5hp</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VGSEA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VIDRG</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>VIDRG</t>
+          <t>VSADA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -595,44 +595,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>`Media och kommunikation inom idrott` (7,5hp); rad: - Media och kommunikation inom idrott, 7,5hp</t>
+          <t>`Personcentrerad vård av personer med demens` (7,5 hp); rad: - Personcentrerad vård av personer med demens, 7,5 hp</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VIDRG</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>VSADA</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>`Personcentrerad vård av personer med demens` (7,5 hp); rad: - Personcentrerad vård av personer med demens, 7,5 hp</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=VSADA</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E7"/>
+  <autoFilter ref="A1:E6"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -644,8 +617,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>